<commit_message>
finalized the new aesthetics options. but the previews need to be fixed.
</commit_message>
<xml_diff>
--- a/StatisticalAnalyzer_Excel_Template.xlsx
+++ b/StatisticalAnalyzer_Excel_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkrumm\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkrumm\Documents\Statistik_dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D0C95D-859B-4DCA-86F1-B5B261F37241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDD4BC1-ADB2-4425-B409-8D683DF2BBD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OneWay" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="48">
   <si>
     <t>Group</t>
   </si>
@@ -565,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -594,18 +594,82 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="B8">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13">
+        <v>2.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>